<commit_message>
feat(m3): M3 baseline — PED v3.0, tests, CI, migrations
- M3 PED sections 18-27 populated
- INDEX.md and 00-document-control.md updated to v3.0
- 60+ tests (unit, integration, E2E) with backend/tests/README.md
- CI workflows (ci.yml, security.yml)
- Registers (defect, technical debt)
- Release evidence (candidate, summary, residual risk, staging, rollback)
- Migrations (001_initial_schema.sql — 9 tables + seed data)
- RTM updated with M3 columns and test IDs
- Repo hygiene: .gitignore (root + backend), SSL detection in db.ts
- Fixed placeholder values in .env.example files
- Controlled changes: M3-01 (Prisma -> pg), M3-02 (Supabase host)
</commit_message>
<xml_diff>
--- a/documents/Requirements_Traceability_Matrix/Requirements_Traceability_Matrix.xlsx
+++ b/documents/Requirements_Traceability_Matrix/Requirements_Traceability_Matrix.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/789919cd20f43bf3/Documentos/2026/October 2026/SEN381/Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\modzu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="289" documentId="8_{76BBB404-1ECA-4E30-9517-C847694D5072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DB04CA8-7507-4D5B-BEBF-67EDE2FC2A06}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036073AB-FF25-4B3A-9284-B918B2A20AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0B8A7918-82A6-460E-9EBF-F9966EF17AB3}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="3" xr2:uid="{0B8A7918-82A6-460E-9EBF-F9966EF17AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="M1" sheetId="3" r:id="rId1"/>
     <sheet name="M2" sheetId="1" r:id="rId2"/>
     <sheet name="M3" sheetId="2" r:id="rId3"/>
+    <sheet name="M3 after testing " sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="471">
   <si>
     <t>Req ID</t>
   </si>
@@ -1173,6 +1174,405 @@
   </si>
   <si>
     <t>Given the system is in production, when availability is measured over a thirty-day period, then uptime must be at least 99.5%during operational hours.</t>
+  </si>
+  <si>
+    <t>Req. ID</t>
+  </si>
+  <si>
+    <t>ACFR-01</t>
+  </si>
+  <si>
+    <t>Given that a citizen opens the report form, when they attach a photo and submit, then the report includes GPS coordinates.</t>
+  </si>
+  <si>
+    <t>Clear work orders, offline capability, status update tools</t>
+  </si>
+  <si>
+    <t>ACFR-02</t>
+  </si>
+  <si>
+    <t>ACFR-03</t>
+  </si>
+  <si>
+    <t>ACFR-04</t>
+  </si>
+  <si>
+    <t>ACFR-05</t>
+  </si>
+  <si>
+    <t>Given a citizen has submitted a report, when the report status changes to Assigned, In Progress, or Resolved, then an alert is sent on the website.</t>
+  </si>
+  <si>
+    <t>ACFR-06</t>
+  </si>
+  <si>
+    <t>ACFR-07</t>
+  </si>
+  <si>
+    <t>Given a field worker is onsite at a job location, when they update a job status, then they must be able to attach at least one photo and enter textual notes as part of the update.</t>
+  </si>
+  <si>
+    <t>ACNFR-01</t>
+  </si>
+  <si>
+    <t>Given a field worker device has been offline with up to twenty cached job card updates, when connectivity is restored, then all updates must be confirmed as synced to the server within less than 10 seconds, with a visible confirmation indicator on the device.</t>
+  </si>
+  <si>
+    <t>ACNFR-02</t>
+  </si>
+  <si>
+    <t>Given one hundred concurrent users are accessing the system during peak hours, when any page is requested, then the median response time across all requests must be under three seconds.</t>
+  </si>
+  <si>
+    <t>ACNFR-03</t>
+  </si>
+  <si>
+    <t>Given a citizen submits a report, when the data is transmitted, then it must be encrypted using HTTPS with TLS as verified by browser security inspection tools.</t>
+  </si>
+  <si>
+    <t>Easy to use interface</t>
+  </si>
+  <si>
+    <t>ACNFR-04</t>
+  </si>
+  <si>
+    <t>ACNFR-05</t>
+  </si>
+  <si>
+    <t>Given the system is in production, when availability is measured over a thirty-day period, then uptime must be at least 99.5% during operational hours.</t>
+  </si>
+  <si>
+    <t>ACFR-08</t>
+  </si>
+  <si>
+    <t>ACFR-09</t>
+  </si>
+  <si>
+    <t>ACFR-10</t>
+  </si>
+  <si>
+    <t>ACFR-11</t>
+  </si>
+  <si>
+    <t>ACFR-12</t>
+  </si>
+  <si>
+    <t>ACFR-13</t>
+  </si>
+  <si>
+    <t>ACFR-14</t>
+  </si>
+  <si>
+    <t>ACFR-15</t>
+  </si>
+  <si>
+    <t>ACNFR-06</t>
+  </si>
+  <si>
+    <t>ACNFR-07</t>
+  </si>
+  <si>
+    <t>ACNFR-08</t>
+  </si>
+  <si>
+    <t>ACNFR-09</t>
+  </si>
+  <si>
+    <t>ACNFR-10</t>
+  </si>
+  <si>
+    <t>ACNFR-11</t>
+  </si>
+  <si>
+    <t>M3 Implementation</t>
+  </si>
+  <si>
+    <t>M3 Test Evidence (IDs)</t>
+  </si>
+  <si>
+    <t>Verified</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-01, TC-BE-REQ-02, TC-BE-REQ-03, TC-BE-REQ-04, TC-E2E-02</t>
+  </si>
+  <si>
+    <t>backend/server/routes/sync.ts</t>
+  </si>
+  <si>
+    <t>(pending sync tests)</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-09</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/requests.test.ts</t>
+  </si>
+  <si>
+    <t>TC-BE-TRANS-01, TC-BE-TRANS-02, TC-BE-TRANS-03, TC-BE-TRANS-04, TC-BE-TRANS-05, TC-BE-TRANS-06, TC-E2E-02</t>
+  </si>
+  <si>
+    <t>TC-BE-TRANS-05</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/transitions.test.ts</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-08</t>
+  </si>
+  <si>
+    <t>(pending field update tests)</t>
+  </si>
+  <si>
+    <t>(pending timing tests)</t>
+  </si>
+  <si>
+    <t>Supabase TLS + PaaS HTTPS (per ADR-TECH-02)</t>
+  </si>
+  <si>
+    <t>Manual verification via browser DevTools</t>
+  </si>
+  <si>
+    <t>Manual viewport check</t>
+  </si>
+  <si>
+    <t>TC-API-01</t>
+  </si>
+  <si>
+    <t>tests/api/health.test.ts</t>
+  </si>
+  <si>
+    <t>TBD (design not yet produced). Constraints: RR074 (pagination), RR114 (ownership checks), RR124 (duplicate-account detection).</t>
+  </si>
+  <si>
+    <t>(pending)</t>
+  </si>
+  <si>
+    <t>TBD (M2 schema design). Constraints: RR075 (indexes), RR108 (role-scoped filtering), RR121 (filter UI).</t>
+  </si>
+  <si>
+    <t>TBD (design not yet produced). Constraints: RR088, RR076, RR122, RR115, RR127, FE006.</t>
+  </si>
+  <si>
+    <t>TC-BE-AUTH-01, TC-BE-AUTH-02, TC-BE-AUTH-03, TC-BE-AUTH-04, TC-BE-AUTH-05, TC-BE-AUTH-06, TC-BE-AUTH-07, TC-BE-AUTH-08, TC-BE-AUTH-09</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/auth.test.ts</t>
+  </si>
+  <si>
+    <t>TBD (M2 stack evaluation). Constraints: RR077, RR109, RR145, RR093.</t>
+  </si>
+  <si>
+    <t>Non-sequential random identifiers (RR110); receipt generated from validated submission data (RR128).</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-01, TC-E2E-02</t>
+  </si>
+  <si>
+    <t>TBD (design not yet produced). Constraints: RR079, RR123, RR119.</t>
+  </si>
+  <si>
+    <t>TC-BE-TRANS-05 (history recorded)</t>
+  </si>
+  <si>
+    <t>TBD (design not yet produced). Constraints: RR086, RR117, RR116, RR072, RR120.</t>
+  </si>
+  <si>
+    <t>TC-BE-AUTH-06, TC-BE-AUTH-07, TC-BE-AUTH-08</t>
+  </si>
+  <si>
+    <t>backend/server/middleware/error.middleware.ts</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-02, TC-BE-REQ-03, TC-BE-REQ-04, TC-BE-TRANS-02, TC-BE-TRANS-04</t>
+  </si>
+  <si>
+    <t>TBD. Constraint: PED Technology Constraint 2.</t>
+  </si>
+  <si>
+    <t>React + Vite build (browser-agnostic)</t>
+  </si>
+  <si>
+    <t>Manual compatibility check</t>
+  </si>
+  <si>
+    <t>Implicit (all tests exercise timestamps)</t>
+  </si>
+  <si>
+    <t>backend/server/persistence/request.repository.ts</t>
+  </si>
+  <si>
+    <t>ADR-CREATE-01; Browser Geolocation/Media APIs. Risks: RR006, RR004.</t>
+  </si>
+  <si>
+    <t>backend/server/routes/requests.ts POST /api/requests</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: implementation + test evidence added; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/requests.test.ts, backend/tests/e2e/admin-resolve.test.ts</t>
+  </si>
+  <si>
+    <t>FE001 technical spike; ADR-PERSIST-01. Risks: RR001, RR132.</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: implementation path identified; tests pending.</t>
+  </si>
+  <si>
+    <t>ADR-CREATE-01; ADR-PERSIST-01; FE006.</t>
+  </si>
+  <si>
+    <t>request.repository.list with department filter</t>
+  </si>
+  <si>
+    <t>ADR-CREATE-01; ADR-PERSIST-01; RBAC Constraint 2. Risks: RR083, RR130, RR122.</t>
+  </si>
+  <si>
+    <t>workflow.service.transition PATCH /api/requests/:id/status</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/transitions.test.ts, backend/tests/e2e/admin-resolve.test.ts</t>
+  </si>
+  <si>
+    <t>ADR-NOTIFY-01; ADR-INT-01; ADR-PERSIST-01. Risks: RR081, RR093.</t>
+  </si>
+  <si>
+    <t>eventBus.raise() post-commit in backend/server/application/workflow.service.ts</t>
+  </si>
+  <si>
+    <t>ADR-NOTIFY-01; ADR-PERSIST-01. Risks: RR110, RR114.</t>
+  </si>
+  <si>
+    <t>GET /api/requests?q= free-text search by tracking number (request.repository.list)</t>
+  </si>
+  <si>
+    <t>ADR-PERSIST-01; Browser Media Capture API. Risks: RR113, RR129.</t>
+  </si>
+  <si>
+    <t>workflow.service.addFieldUpdate POST /api/requests/:id/update</t>
+  </si>
+  <si>
+    <t>FE001 spike and conflict strategy (ADR-PERSIST-01); PED Quality Constraint 2. Risk: RR001.</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: implementation path identified; timing tests pending.</t>
+  </si>
+  <si>
+    <t>ADR-PERSIST-01 caching position; Indexing and query optimisation (Quality Constraint 3; FE006). Risks: RR005, RR074–RR076.</t>
+  </si>
+  <si>
+    <t>Layered API + indexed DB (backend/server/index.ts, request.repository.ts)</t>
+  </si>
+  <si>
+    <t>Performance test tests/performance/load-test.js (placeholder)</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: performance test script placeholder; load test pending.</t>
+  </si>
+  <si>
+    <t>PED Security Constraint 1 (HTTPS/TLS, encryption at rest, POPIA); Supabase TLS + PaaS HTTPS (per ADR-TECH-02).</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: stack-level verification confirmed; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>ADR-TECH-02, documents/Architecture_Decision_Record/</t>
+  </si>
+  <si>
+    <t>ED-002 (single web-responsive codebase); Technology Constraint 2 (CSS media queries). Risk: RR120.</t>
+  </si>
+  <si>
+    <t>React responsive components in frontend/src/</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: implementation in place; verification pending.</t>
+  </si>
+  <si>
+    <t>FE003 (hosting path, free-tier limits), FE004 (monitoring), FE005 (backup and recovery). Risk: RR094.</t>
+  </si>
+  <si>
+    <t>Health endpoint (backend/server/index.ts /health) + stateless service</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: health endpoint verified; production monitoring pending.</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: unchanged.</t>
+  </si>
+  <si>
+    <t>Municipal Field Workers/Administrators</t>
+  </si>
+  <si>
+    <t>ADR-PERSIST-01: assignment change inside the status-transition transaction; optimistic concurrency (version column). Risks: RR083, RR122, RR125, RR156.</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: implementation + test evidence added; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>Analytics dashboards, performance reporting</t>
+  </si>
+  <si>
+    <t>The system shall allow users to register and authenticate (citizen and staff accounts).</t>
+  </si>
+  <si>
+    <t>Established auth and hashing libraries (bcryptjs, jsonwebtoken). Constraints: RR112, RR144, RR104, RR130, RR111, RR124, RR133, RR134, RR135, RR139.</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: implementation + 9 tests added; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>GPS locations</t>
+  </si>
+  <si>
+    <t>POST /api/requests returns trackingNumber in response</t>
+  </si>
+  <si>
+    <t>ADR-PERSIST-01: append-only history/audit table; corrections recorded as new entries. Constraints: RR137, RR087, RR107, RR136, RR078, RR139.</t>
+  </si>
+  <si>
+    <t>request_history table in backend/server/persistence/request.repository.ts</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: append-only history implemented; retention policy pending.</t>
+  </si>
+  <si>
+    <t>JWT with expiry (JWT_EXPIRES_IN = "8h" in routes/auth.ts). Constraints: RR131, RR105, RR132.</t>
+  </si>
+  <si>
+    <t>routes/auth.ts jwt.sign(..., { expiresIn: JWT_EXPIRES_IN })</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: JWT expiry verified via auth tests; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>Centralised error-handling layer (asyncHandler, HttpError in middleware/error.middleware.ts). Constraints: RR084, RR103.</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: error handler verified via negative tests; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/requests.test.ts, backend/tests/integration/transitions.test.ts</t>
+  </si>
+  <si>
+    <t>Postgres now() stores UTC; request_history.at uses now() default. Constraints: RR127, RR085, RR069, RR092.</t>
+  </si>
+  <si>
+    <t>backend/server/persistence/request.repository.ts UTC storage via now()</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: UTC storage verified; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>workflow.service.acceptJob  - POST /api/requests/:id/accept</t>
+  </si>
+  <si>
+    <t>routes/auth.ts - POST /api/auth/login, POST /api/auth/logout, GET /api/auth/me</t>
+  </si>
+  <si>
+    <t>(accept endpoint not yet tested)</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: implementation path identified; accept endpoint tests pending.</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1726,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1352,17 +1752,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1371,7 +1764,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1712,497 +2104,497 @@
     <col min="1" max="12" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="16" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="12" t="s">
         <v>285</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="12" t="s">
         <v>288</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="12" t="s">
         <v>289</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="K1" s="12" t="s">
         <v>291</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="L1" s="12" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I2" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J2" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K2" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L2" s="13" t="s">
+      <c r="I2" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I3" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J3" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K3" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L3" s="13" t="s">
+      <c r="I3" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L3" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="10" t="s">
         <v>307</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I4" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K4" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L4" s="13" t="s">
+      <c r="I4" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L4" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="10" t="s">
         <v>310</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I5" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L5" s="13" t="s">
+      <c r="I5" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L5" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="10" t="s">
         <v>312</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I6" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J6" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K6" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L6" s="13" t="s">
+      <c r="I6" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L6" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G7" s="10" t="s">
         <v>316</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="H7" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I7" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K7" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L7" s="13" t="s">
+      <c r="I7" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L7" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I8" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J8" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K8" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L8" s="13" t="s">
+      <c r="I8" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L8" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="10" t="s">
         <v>322</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I9" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L9" s="13" t="s">
+      <c r="I9" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L9" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="87" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I10" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J10" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K10" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L10" s="13" t="s">
+      <c r="I10" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L10" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="10" t="s">
         <v>329</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I11" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J11" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L11" s="13" t="s">
+      <c r="I11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L11" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="87" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="10" t="s">
         <v>331</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="10" t="s">
         <v>332</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I12" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J12" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K12" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L12" s="13" t="s">
+      <c r="I12" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L12" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="10" t="s">
         <v>334</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="10" t="s">
         <v>335</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="G13" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="H13" s="13" t="s">
+      <c r="H13" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I13" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J13" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K13" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L13" s="13" t="s">
+      <c r="I13" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L13" s="10" t="s">
         <v>232</v>
       </c>
     </row>
@@ -2218,11 +2610,10 @@
   <cols>
     <col min="1" max="1" width="30.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.77734375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="30.77734375" style="11" customWidth="1"/>
-    <col min="4" max="13" width="30.77734375" customWidth="1"/>
+    <col min="3" max="13" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="9" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2263,14 +2654,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -2304,14 +2695,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -2345,14 +2736,14 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" s="3" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -2386,14 +2777,14 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="4" t="s">
         <v>93</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -2427,14 +2818,14 @@
         <v>256</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" s="3" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -2468,14 +2859,14 @@
         <v>257</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -2509,14 +2900,14 @@
         <v>258</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -2550,14 +2941,14 @@
         <v>259</v>
       </c>
     </row>
-    <row r="9" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -2591,14 +2982,14 @@
         <v>260</v>
       </c>
     </row>
-    <row r="10" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -2632,14 +3023,14 @@
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:13" s="3" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="4" t="s">
         <v>279</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -2673,14 +3064,14 @@
         <v>262</v>
       </c>
     </row>
-    <row r="12" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -2714,14 +3105,14 @@
         <v>263</v>
       </c>
     </row>
-    <row r="13" spans="1:13" s="3" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="4" t="s">
         <v>281</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -2755,7 +3146,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="14" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>24</v>
       </c>
@@ -2796,7 +3187,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>25</v>
       </c>
@@ -2837,7 +3228,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>26</v>
       </c>
@@ -2878,7 +3269,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="17" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>27</v>
       </c>
@@ -2919,7 +3310,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>28</v>
       </c>
@@ -2960,7 +3351,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="19" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>29</v>
       </c>
@@ -3001,7 +3392,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>30</v>
       </c>
@@ -3042,7 +3433,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="21" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>31</v>
       </c>
@@ -3083,7 +3474,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="22" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
@@ -3124,7 +3515,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="23" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
@@ -3165,7 +3556,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="24" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
@@ -3206,7 +3597,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>35</v>
       </c>
@@ -3247,7 +3638,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="26" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>36</v>
       </c>
@@ -3288,7 +3679,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="27" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>37</v>
       </c>
@@ -3394,7 +3785,7 @@
       <c r="B2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -3435,7 +3826,7 @@
       <c r="B3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -3476,7 +3867,7 @@
       <c r="B4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -3517,7 +3908,7 @@
       <c r="B5" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="4" t="s">
         <v>93</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -3558,7 +3949,7 @@
       <c r="B6" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -3599,7 +3990,7 @@
       <c r="B7" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -3640,7 +4031,7 @@
       <c r="B8" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -3681,7 +4072,7 @@
       <c r="B9" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -3722,7 +4113,7 @@
       <c r="B10" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -3763,7 +4154,7 @@
       <c r="B11" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="4" t="s">
         <v>279</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -3804,7 +4195,7 @@
       <c r="B12" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -3845,7 +4236,7 @@
       <c r="B13" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="4" t="s">
         <v>281</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -4289,7 +4680,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
@@ -4452,6 +4843,1152 @@
       <c r="M27" s="4" t="s">
         <v>278</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43033B97-8DA6-4871-83EC-7EBCF2C2C0E3}">
+  <dimension ref="A1:N27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="13" width="30.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="N2" s="4"/>
+    </row>
+    <row r="3" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N3" s="4"/>
+    </row>
+    <row r="4" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="N4" s="4"/>
+    </row>
+    <row r="5" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="N5" s="4"/>
+    </row>
+    <row r="6" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="N6" s="4"/>
+    </row>
+    <row r="7" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="N7" s="4"/>
+    </row>
+    <row r="8" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N8" s="4"/>
+    </row>
+    <row r="9" spans="1:14" ht="92.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N9" s="4"/>
+    </row>
+    <row r="10" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N10" s="4"/>
+    </row>
+    <row r="11" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="N11" s="4"/>
+    </row>
+    <row r="12" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N12" s="4"/>
+    </row>
+    <row r="13" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N13" s="4"/>
+    </row>
+    <row r="14" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N14" s="4"/>
+    </row>
+    <row r="15" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N15" s="4"/>
+    </row>
+    <row r="16" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="N16" s="4"/>
+    </row>
+    <row r="17" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N17" s="4"/>
+    </row>
+    <row r="18" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="N18" s="4"/>
+    </row>
+    <row r="19" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M19" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N19" s="4"/>
+    </row>
+    <row r="20" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="N20" s="4"/>
+    </row>
+    <row r="21" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N21" s="4"/>
+    </row>
+    <row r="22" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="M22" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="N22" s="4"/>
+    </row>
+    <row r="23" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N23" s="4"/>
+    </row>
+    <row r="24" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="N24" s="4"/>
+    </row>
+    <row r="25" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="N25" s="4"/>
+    </row>
+    <row r="26" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N26" s="4"/>
+    </row>
+    <row r="27" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="N27" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs(m4): move all documentation from SRC-UPDATE to Documentation branch
</commit_message>
<xml_diff>
--- a/documents/Requirements_Traceability_Matrix/Requirements_Traceability_Matrix.xlsx
+++ b/documents/Requirements_Traceability_Matrix/Requirements_Traceability_Matrix.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/789919cd20f43bf3/Documentos/2026/October 2026/SEN381/Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\modzu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="289" documentId="8_{76BBB404-1ECA-4E30-9517-C847694D5072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DB04CA8-7507-4D5B-BEBF-67EDE2FC2A06}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036073AB-FF25-4B3A-9284-B918B2A20AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0B8A7918-82A6-460E-9EBF-F9966EF17AB3}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="3" xr2:uid="{0B8A7918-82A6-460E-9EBF-F9966EF17AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="M1" sheetId="3" r:id="rId1"/>
     <sheet name="M2" sheetId="1" r:id="rId2"/>
     <sheet name="M3" sheetId="2" r:id="rId3"/>
+    <sheet name="M3 after testing " sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="471">
   <si>
     <t>Req ID</t>
   </si>
@@ -1173,6 +1174,405 @@
   </si>
   <si>
     <t>Given the system is in production, when availability is measured over a thirty-day period, then uptime must be at least 99.5%during operational hours.</t>
+  </si>
+  <si>
+    <t>Req. ID</t>
+  </si>
+  <si>
+    <t>ACFR-01</t>
+  </si>
+  <si>
+    <t>Given that a citizen opens the report form, when they attach a photo and submit, then the report includes GPS coordinates.</t>
+  </si>
+  <si>
+    <t>Clear work orders, offline capability, status update tools</t>
+  </si>
+  <si>
+    <t>ACFR-02</t>
+  </si>
+  <si>
+    <t>ACFR-03</t>
+  </si>
+  <si>
+    <t>ACFR-04</t>
+  </si>
+  <si>
+    <t>ACFR-05</t>
+  </si>
+  <si>
+    <t>Given a citizen has submitted a report, when the report status changes to Assigned, In Progress, or Resolved, then an alert is sent on the website.</t>
+  </si>
+  <si>
+    <t>ACFR-06</t>
+  </si>
+  <si>
+    <t>ACFR-07</t>
+  </si>
+  <si>
+    <t>Given a field worker is onsite at a job location, when they update a job status, then they must be able to attach at least one photo and enter textual notes as part of the update.</t>
+  </si>
+  <si>
+    <t>ACNFR-01</t>
+  </si>
+  <si>
+    <t>Given a field worker device has been offline with up to twenty cached job card updates, when connectivity is restored, then all updates must be confirmed as synced to the server within less than 10 seconds, with a visible confirmation indicator on the device.</t>
+  </si>
+  <si>
+    <t>ACNFR-02</t>
+  </si>
+  <si>
+    <t>Given one hundred concurrent users are accessing the system during peak hours, when any page is requested, then the median response time across all requests must be under three seconds.</t>
+  </si>
+  <si>
+    <t>ACNFR-03</t>
+  </si>
+  <si>
+    <t>Given a citizen submits a report, when the data is transmitted, then it must be encrypted using HTTPS with TLS as verified by browser security inspection tools.</t>
+  </si>
+  <si>
+    <t>Easy to use interface</t>
+  </si>
+  <si>
+    <t>ACNFR-04</t>
+  </si>
+  <si>
+    <t>ACNFR-05</t>
+  </si>
+  <si>
+    <t>Given the system is in production, when availability is measured over a thirty-day period, then uptime must be at least 99.5% during operational hours.</t>
+  </si>
+  <si>
+    <t>ACFR-08</t>
+  </si>
+  <si>
+    <t>ACFR-09</t>
+  </si>
+  <si>
+    <t>ACFR-10</t>
+  </si>
+  <si>
+    <t>ACFR-11</t>
+  </si>
+  <si>
+    <t>ACFR-12</t>
+  </si>
+  <si>
+    <t>ACFR-13</t>
+  </si>
+  <si>
+    <t>ACFR-14</t>
+  </si>
+  <si>
+    <t>ACFR-15</t>
+  </si>
+  <si>
+    <t>ACNFR-06</t>
+  </si>
+  <si>
+    <t>ACNFR-07</t>
+  </si>
+  <si>
+    <t>ACNFR-08</t>
+  </si>
+  <si>
+    <t>ACNFR-09</t>
+  </si>
+  <si>
+    <t>ACNFR-10</t>
+  </si>
+  <si>
+    <t>ACNFR-11</t>
+  </si>
+  <si>
+    <t>M3 Implementation</t>
+  </si>
+  <si>
+    <t>M3 Test Evidence (IDs)</t>
+  </si>
+  <si>
+    <t>Verified</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-01, TC-BE-REQ-02, TC-BE-REQ-03, TC-BE-REQ-04, TC-E2E-02</t>
+  </si>
+  <si>
+    <t>backend/server/routes/sync.ts</t>
+  </si>
+  <si>
+    <t>(pending sync tests)</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-09</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/requests.test.ts</t>
+  </si>
+  <si>
+    <t>TC-BE-TRANS-01, TC-BE-TRANS-02, TC-BE-TRANS-03, TC-BE-TRANS-04, TC-BE-TRANS-05, TC-BE-TRANS-06, TC-E2E-02</t>
+  </si>
+  <si>
+    <t>TC-BE-TRANS-05</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/transitions.test.ts</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-08</t>
+  </si>
+  <si>
+    <t>(pending field update tests)</t>
+  </si>
+  <si>
+    <t>(pending timing tests)</t>
+  </si>
+  <si>
+    <t>Supabase TLS + PaaS HTTPS (per ADR-TECH-02)</t>
+  </si>
+  <si>
+    <t>Manual verification via browser DevTools</t>
+  </si>
+  <si>
+    <t>Manual viewport check</t>
+  </si>
+  <si>
+    <t>TC-API-01</t>
+  </si>
+  <si>
+    <t>tests/api/health.test.ts</t>
+  </si>
+  <si>
+    <t>TBD (design not yet produced). Constraints: RR074 (pagination), RR114 (ownership checks), RR124 (duplicate-account detection).</t>
+  </si>
+  <si>
+    <t>(pending)</t>
+  </si>
+  <si>
+    <t>TBD (M2 schema design). Constraints: RR075 (indexes), RR108 (role-scoped filtering), RR121 (filter UI).</t>
+  </si>
+  <si>
+    <t>TBD (design not yet produced). Constraints: RR088, RR076, RR122, RR115, RR127, FE006.</t>
+  </si>
+  <si>
+    <t>TC-BE-AUTH-01, TC-BE-AUTH-02, TC-BE-AUTH-03, TC-BE-AUTH-04, TC-BE-AUTH-05, TC-BE-AUTH-06, TC-BE-AUTH-07, TC-BE-AUTH-08, TC-BE-AUTH-09</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/auth.test.ts</t>
+  </si>
+  <si>
+    <t>TBD (M2 stack evaluation). Constraints: RR077, RR109, RR145, RR093.</t>
+  </si>
+  <si>
+    <t>Non-sequential random identifiers (RR110); receipt generated from validated submission data (RR128).</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-01, TC-E2E-02</t>
+  </si>
+  <si>
+    <t>TBD (design not yet produced). Constraints: RR079, RR123, RR119.</t>
+  </si>
+  <si>
+    <t>TC-BE-TRANS-05 (history recorded)</t>
+  </si>
+  <si>
+    <t>TBD (design not yet produced). Constraints: RR086, RR117, RR116, RR072, RR120.</t>
+  </si>
+  <si>
+    <t>TC-BE-AUTH-06, TC-BE-AUTH-07, TC-BE-AUTH-08</t>
+  </si>
+  <si>
+    <t>backend/server/middleware/error.middleware.ts</t>
+  </si>
+  <si>
+    <t>TC-BE-REQ-02, TC-BE-REQ-03, TC-BE-REQ-04, TC-BE-TRANS-02, TC-BE-TRANS-04</t>
+  </si>
+  <si>
+    <t>TBD. Constraint: PED Technology Constraint 2.</t>
+  </si>
+  <si>
+    <t>React + Vite build (browser-agnostic)</t>
+  </si>
+  <si>
+    <t>Manual compatibility check</t>
+  </si>
+  <si>
+    <t>Implicit (all tests exercise timestamps)</t>
+  </si>
+  <si>
+    <t>backend/server/persistence/request.repository.ts</t>
+  </si>
+  <si>
+    <t>ADR-CREATE-01; Browser Geolocation/Media APIs. Risks: RR006, RR004.</t>
+  </si>
+  <si>
+    <t>backend/server/routes/requests.ts POST /api/requests</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: implementation + test evidence added; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/requests.test.ts, backend/tests/e2e/admin-resolve.test.ts</t>
+  </si>
+  <si>
+    <t>FE001 technical spike; ADR-PERSIST-01. Risks: RR001, RR132.</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: implementation path identified; tests pending.</t>
+  </si>
+  <si>
+    <t>ADR-CREATE-01; ADR-PERSIST-01; FE006.</t>
+  </si>
+  <si>
+    <t>request.repository.list with department filter</t>
+  </si>
+  <si>
+    <t>ADR-CREATE-01; ADR-PERSIST-01; RBAC Constraint 2. Risks: RR083, RR130, RR122.</t>
+  </si>
+  <si>
+    <t>workflow.service.transition PATCH /api/requests/:id/status</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/transitions.test.ts, backend/tests/e2e/admin-resolve.test.ts</t>
+  </si>
+  <si>
+    <t>ADR-NOTIFY-01; ADR-INT-01; ADR-PERSIST-01. Risks: RR081, RR093.</t>
+  </si>
+  <si>
+    <t>eventBus.raise() post-commit in backend/server/application/workflow.service.ts</t>
+  </si>
+  <si>
+    <t>ADR-NOTIFY-01; ADR-PERSIST-01. Risks: RR110, RR114.</t>
+  </si>
+  <si>
+    <t>GET /api/requests?q= free-text search by tracking number (request.repository.list)</t>
+  </si>
+  <si>
+    <t>ADR-PERSIST-01; Browser Media Capture API. Risks: RR113, RR129.</t>
+  </si>
+  <si>
+    <t>workflow.service.addFieldUpdate POST /api/requests/:id/update</t>
+  </si>
+  <si>
+    <t>FE001 spike and conflict strategy (ADR-PERSIST-01); PED Quality Constraint 2. Risk: RR001.</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: implementation path identified; timing tests pending.</t>
+  </si>
+  <si>
+    <t>ADR-PERSIST-01 caching position; Indexing and query optimisation (Quality Constraint 3; FE006). Risks: RR005, RR074–RR076.</t>
+  </si>
+  <si>
+    <t>Layered API + indexed DB (backend/server/index.ts, request.repository.ts)</t>
+  </si>
+  <si>
+    <t>Performance test tests/performance/load-test.js (placeholder)</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: performance test script placeholder; load test pending.</t>
+  </si>
+  <si>
+    <t>PED Security Constraint 1 (HTTPS/TLS, encryption at rest, POPIA); Supabase TLS + PaaS HTTPS (per ADR-TECH-02).</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: stack-level verification confirmed; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>ADR-TECH-02, documents/Architecture_Decision_Record/</t>
+  </si>
+  <si>
+    <t>ED-002 (single web-responsive codebase); Technology Constraint 2 (CSS media queries). Risk: RR120.</t>
+  </si>
+  <si>
+    <t>React responsive components in frontend/src/</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: implementation in place; verification pending.</t>
+  </si>
+  <si>
+    <t>FE003 (hosting path, free-tier limits), FE004 (monitoring), FE005 (backup and recovery). Risk: RR094.</t>
+  </si>
+  <si>
+    <t>Health endpoint (backend/server/index.ts /health) + stateless service</t>
+  </si>
+  <si>
+    <t>v1.0: baselined. v2.0: Design Link, planned tests, risks added. v3.0: health endpoint verified; production monitoring pending.</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: unchanged.</t>
+  </si>
+  <si>
+    <t>Municipal Field Workers/Administrators</t>
+  </si>
+  <si>
+    <t>ADR-PERSIST-01: assignment change inside the status-transition transaction; optimistic concurrency (version column). Risks: RR083, RR122, RR125, RR156.</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: implementation + test evidence added; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>Analytics dashboards, performance reporting</t>
+  </si>
+  <si>
+    <t>The system shall allow users to register and authenticate (citizen and staff accounts).</t>
+  </si>
+  <si>
+    <t>Established auth and hashing libraries (bcryptjs, jsonwebtoken). Constraints: RR112, RR144, RR104, RR130, RR111, RR124, RR133, RR134, RR135, RR139.</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: implementation + 9 tests added; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>GPS locations</t>
+  </si>
+  <si>
+    <t>POST /api/requests returns trackingNumber in response</t>
+  </si>
+  <si>
+    <t>ADR-PERSIST-01: append-only history/audit table; corrections recorded as new entries. Constraints: RR137, RR087, RR107, RR136, RR078, RR139.</t>
+  </si>
+  <si>
+    <t>request_history table in backend/server/persistence/request.repository.ts</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: append-only history implemented; retention policy pending.</t>
+  </si>
+  <si>
+    <t>JWT with expiry (JWT_EXPIRES_IN = "8h" in routes/auth.ts). Constraints: RR131, RR105, RR132.</t>
+  </si>
+  <si>
+    <t>routes/auth.ts jwt.sign(..., { expiresIn: JWT_EXPIRES_IN })</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: JWT expiry verified via auth tests; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>Centralised error-handling layer (asyncHandler, HttpError in middleware/error.middleware.ts). Constraints: RR084, RR103.</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: error handler verified via negative tests; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>backend/tests/integration/requests.test.ts, backend/tests/integration/transitions.test.ts</t>
+  </si>
+  <si>
+    <t>Postgres now() stores UTC; request_history.at uses now() default. Constraints: RR127, RR085, RR069, RR092.</t>
+  </si>
+  <si>
+    <t>backend/server/persistence/request.repository.ts UTC storage via now()</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: UTC storage verified; status -&gt; Verified.</t>
+  </si>
+  <si>
+    <t>workflow.service.acceptJob  - POST /api/requests/:id/accept</t>
+  </si>
+  <si>
+    <t>routes/auth.ts - POST /api/auth/login, POST /api/auth/logout, GET /api/auth/me</t>
+  </si>
+  <si>
+    <t>(accept endpoint not yet tested)</t>
+  </si>
+  <si>
+    <t>v2.0: added. v3.0: implementation path identified; accept endpoint tests pending.</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1726,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1352,17 +1752,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1371,7 +1764,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1712,497 +2104,497 @@
     <col min="1" max="12" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="16" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="12" t="s">
         <v>285</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="12" t="s">
         <v>288</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="12" t="s">
         <v>289</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="K1" s="12" t="s">
         <v>291</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="L1" s="12" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I2" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J2" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K2" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L2" s="13" t="s">
+      <c r="I2" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I3" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J3" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K3" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L3" s="13" t="s">
+      <c r="I3" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L3" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="10" t="s">
         <v>307</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I4" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K4" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L4" s="13" t="s">
+      <c r="I4" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L4" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="10" t="s">
         <v>310</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I5" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L5" s="13" t="s">
+      <c r="I5" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L5" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="10" t="s">
         <v>312</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I6" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J6" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K6" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L6" s="13" t="s">
+      <c r="I6" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L6" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G7" s="10" t="s">
         <v>316</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="H7" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I7" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K7" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L7" s="13" t="s">
+      <c r="I7" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L7" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I8" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J8" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K8" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L8" s="13" t="s">
+      <c r="I8" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L8" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="10" t="s">
         <v>322</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I9" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L9" s="13" t="s">
+      <c r="I9" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L9" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="87" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I10" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J10" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K10" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L10" s="13" t="s">
+      <c r="I10" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L10" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="10" t="s">
         <v>329</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I11" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J11" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L11" s="13" t="s">
+      <c r="I11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L11" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="87" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="10" t="s">
         <v>314</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="10" t="s">
         <v>331</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="10" t="s">
         <v>332</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I12" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J12" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K12" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L12" s="13" t="s">
+      <c r="I12" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L12" s="10" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="10" t="s">
         <v>334</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="10" t="s">
         <v>335</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="G13" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="H13" s="13" t="s">
+      <c r="H13" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="I13" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="J13" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="K13" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="L13" s="13" t="s">
+      <c r="I13" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L13" s="10" t="s">
         <v>232</v>
       </c>
     </row>
@@ -2218,11 +2610,10 @@
   <cols>
     <col min="1" max="1" width="30.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.77734375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="30.77734375" style="11" customWidth="1"/>
-    <col min="4" max="13" width="30.77734375" customWidth="1"/>
+    <col min="3" max="13" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="9" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2263,14 +2654,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -2304,14 +2695,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -2345,14 +2736,14 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" s="3" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -2386,14 +2777,14 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="4" t="s">
         <v>93</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -2427,14 +2818,14 @@
         <v>256</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" s="3" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -2468,14 +2859,14 @@
         <v>257</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -2509,14 +2900,14 @@
         <v>258</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -2550,14 +2941,14 @@
         <v>259</v>
       </c>
     </row>
-    <row r="9" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -2591,14 +2982,14 @@
         <v>260</v>
       </c>
     </row>
-    <row r="10" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -2632,14 +3023,14 @@
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:13" s="3" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="4" t="s">
         <v>279</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -2673,14 +3064,14 @@
         <v>262</v>
       </c>
     </row>
-    <row r="12" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -2714,14 +3105,14 @@
         <v>263</v>
       </c>
     </row>
-    <row r="13" spans="1:13" s="3" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="4" t="s">
         <v>281</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -2755,7 +3146,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="14" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>24</v>
       </c>
@@ -2796,7 +3187,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>25</v>
       </c>
@@ -2837,7 +3228,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>26</v>
       </c>
@@ -2878,7 +3269,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="17" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>27</v>
       </c>
@@ -2919,7 +3310,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>28</v>
       </c>
@@ -2960,7 +3351,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="19" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>29</v>
       </c>
@@ -3001,7 +3392,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>30</v>
       </c>
@@ -3042,7 +3433,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="21" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" s="3" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>31</v>
       </c>
@@ -3083,7 +3474,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="22" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
@@ -3124,7 +3515,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="23" spans="1:13" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
@@ -3165,7 +3556,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="24" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
@@ -3206,7 +3597,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>35</v>
       </c>
@@ -3247,7 +3638,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="26" spans="1:13" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>36</v>
       </c>
@@ -3288,7 +3679,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="27" spans="1:13" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>37</v>
       </c>
@@ -3394,7 +3785,7 @@
       <c r="B2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -3435,7 +3826,7 @@
       <c r="B3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -3476,7 +3867,7 @@
       <c r="B4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -3517,7 +3908,7 @@
       <c r="B5" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="4" t="s">
         <v>93</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -3558,7 +3949,7 @@
       <c r="B6" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -3599,7 +3990,7 @@
       <c r="B7" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -3640,7 +4031,7 @@
       <c r="B8" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -3681,7 +4072,7 @@
       <c r="B9" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -3722,7 +4113,7 @@
       <c r="B10" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -3763,7 +4154,7 @@
       <c r="B11" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="4" t="s">
         <v>279</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -3804,7 +4195,7 @@
       <c r="B12" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -3845,7 +4236,7 @@
       <c r="B13" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="4" t="s">
         <v>281</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -4289,7 +4680,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
@@ -4452,6 +4843,1152 @@
       <c r="M27" s="4" t="s">
         <v>278</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43033B97-8DA6-4871-83EC-7EBCF2C2C0E3}">
+  <dimension ref="A1:N27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="13" width="30.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="N2" s="4"/>
+    </row>
+    <row r="3" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N3" s="4"/>
+    </row>
+    <row r="4" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="N4" s="4"/>
+    </row>
+    <row r="5" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="N5" s="4"/>
+    </row>
+    <row r="6" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="N6" s="4"/>
+    </row>
+    <row r="7" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="N7" s="4"/>
+    </row>
+    <row r="8" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N8" s="4"/>
+    </row>
+    <row r="9" spans="1:14" ht="92.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N9" s="4"/>
+    </row>
+    <row r="10" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N10" s="4"/>
+    </row>
+    <row r="11" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="N11" s="4"/>
+    </row>
+    <row r="12" spans="1:14" ht="66" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N12" s="4"/>
+    </row>
+    <row r="13" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N13" s="4"/>
+    </row>
+    <row r="14" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N14" s="4"/>
+    </row>
+    <row r="15" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N15" s="4"/>
+    </row>
+    <row r="16" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="N16" s="4"/>
+    </row>
+    <row r="17" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N17" s="4"/>
+    </row>
+    <row r="18" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="N18" s="4"/>
+    </row>
+    <row r="19" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M19" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N19" s="4"/>
+    </row>
+    <row r="20" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="N20" s="4"/>
+    </row>
+    <row r="21" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N21" s="4"/>
+    </row>
+    <row r="22" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="M22" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="N22" s="4"/>
+    </row>
+    <row r="23" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N23" s="4"/>
+    </row>
+    <row r="24" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="N24" s="4"/>
+    </row>
+    <row r="25" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="N25" s="4"/>
+    </row>
+    <row r="26" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="N26" s="4"/>
+    </row>
+    <row r="27" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="N27" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>